<commit_message>
Primeira versão do apontamento
</commit_message>
<xml_diff>
--- a/modelos/apontamento_manha.xlsx
+++ b/modelos/apontamento_manha.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{5CF2130B-03D7-4201-A06E-E31242A6816B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E0A6F45-10BA-4084-A206-CB34ACB16D10}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{5CF2130B-03D7-4201-A06E-E31242A6816B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{863DF637-E67F-4125-AFAC-C3AD3DDD928C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{18B97131-922C-4537-B241-F72155183AFA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -93,18 +93,6 @@
   </si>
   <si>
     <t>PEDIDO DE VENDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meta: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operador: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Máq: </t>
   </si>
   <si>
     <t>APONTAMENTO DE PRODUÇÃO - NOITE</t>
@@ -190,7 +178,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -647,11 +635,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -702,6 +703,27 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -753,6 +775,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -807,23 +838,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1215,7 +1231,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="11.7109375" customWidth="1"/>
@@ -1238,33 +1254,25 @@
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:18" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="31" t="s">
+      <c r="A2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="32"/>
-      <c r="L2" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="M2" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="N2" s="32"/>
-      <c r="O2" s="67" t="s">
-        <v>22</v>
-      </c>
-      <c r="P2" s="66"/>
-      <c r="Q2" s="68"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="39"/>
+      <c r="O2" s="52"/>
+      <c r="P2" s="53"/>
+      <c r="Q2" s="54"/>
       <c r="R2" s="17"/>
     </row>
     <row r="3" spans="1:18" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1274,14 +1282,14 @@
       <c r="B3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="34"/>
-      <c r="E3" s="33" t="s">
+      <c r="D3" s="41"/>
+      <c r="E3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="34"/>
+      <c r="F3" s="41"/>
       <c r="G3" s="14" t="s">
         <v>2</v>
       </c>
@@ -1306,20 +1314,20 @@
       <c r="N3" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="O3" s="39" t="s">
+      <c r="O3" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="P3" s="39"/>
-      <c r="Q3" s="40"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="47"/>
       <c r="R3" s="19"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="12"/>
       <c r="B4" s="23"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="36"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="43"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
@@ -1328,18 +1336,18 @@
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
-      <c r="O4" s="41"/>
-      <c r="P4" s="41"/>
-      <c r="Q4" s="42"/>
+      <c r="O4" s="48"/>
+      <c r="P4" s="48"/>
+      <c r="Q4" s="49"/>
       <c r="R4" s="18"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="24"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="38"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="45"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1348,18 +1356,18 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
-      <c r="O5" s="43"/>
-      <c r="P5" s="43"/>
-      <c r="Q5" s="44"/>
+      <c r="O5" s="50"/>
+      <c r="P5" s="50"/>
+      <c r="Q5" s="51"/>
       <c r="R5" s="18"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="24"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="38"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="45"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -1368,18 +1376,18 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
-      <c r="O6" s="43"/>
-      <c r="P6" s="43"/>
-      <c r="Q6" s="44"/>
+      <c r="O6" s="50"/>
+      <c r="P6" s="50"/>
+      <c r="Q6" s="51"/>
       <c r="R6" s="18"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="24"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="38"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="45"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -1388,18 +1396,18 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
-      <c r="O7" s="43"/>
-      <c r="P7" s="43"/>
-      <c r="Q7" s="44"/>
+      <c r="O7" s="50"/>
+      <c r="P7" s="50"/>
+      <c r="Q7" s="51"/>
       <c r="R7" s="18"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="24"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="38"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="45"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -1408,18 +1416,18 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
-      <c r="O8" s="43"/>
-      <c r="P8" s="43"/>
-      <c r="Q8" s="44"/>
+      <c r="O8" s="50"/>
+      <c r="P8" s="50"/>
+      <c r="Q8" s="51"/>
       <c r="R8" s="18"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="24"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="38"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="45"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -1428,18 +1436,18 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
-      <c r="O9" s="43"/>
-      <c r="P9" s="43"/>
-      <c r="Q9" s="44"/>
+      <c r="O9" s="50"/>
+      <c r="P9" s="50"/>
+      <c r="Q9" s="51"/>
       <c r="R9" s="18"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="24"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="38"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="45"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -1448,18 +1456,18 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
-      <c r="O10" s="43"/>
-      <c r="P10" s="43"/>
-      <c r="Q10" s="44"/>
+      <c r="O10" s="50"/>
+      <c r="P10" s="50"/>
+      <c r="Q10" s="51"/>
       <c r="R10" s="18"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="24"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="38"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="45"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -1468,18 +1476,18 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
-      <c r="O11" s="43"/>
-      <c r="P11" s="43"/>
-      <c r="Q11" s="44"/>
+      <c r="O11" s="50"/>
+      <c r="P11" s="50"/>
+      <c r="Q11" s="51"/>
       <c r="R11" s="18"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="24"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="38"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="45"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="45"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
@@ -1488,18 +1496,18 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
-      <c r="O12" s="43"/>
-      <c r="P12" s="43"/>
-      <c r="Q12" s="44"/>
+      <c r="O12" s="50"/>
+      <c r="P12" s="50"/>
+      <c r="Q12" s="51"/>
       <c r="R12" s="18"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="24"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="38"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="45"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -1508,18 +1516,18 @@
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
-      <c r="O13" s="43"/>
-      <c r="P13" s="43"/>
-      <c r="Q13" s="44"/>
+      <c r="O13" s="50"/>
+      <c r="P13" s="50"/>
+      <c r="Q13" s="51"/>
       <c r="R13" s="18"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="24"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="38"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="45"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -1528,18 +1536,18 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
-      <c r="O14" s="43"/>
-      <c r="P14" s="43"/>
-      <c r="Q14" s="44"/>
+      <c r="O14" s="50"/>
+      <c r="P14" s="50"/>
+      <c r="Q14" s="51"/>
       <c r="R14" s="18"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="24"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="38"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="45"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -1548,18 +1556,18 @@
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
-      <c r="O15" s="43"/>
-      <c r="P15" s="43"/>
-      <c r="Q15" s="44"/>
+      <c r="O15" s="50"/>
+      <c r="P15" s="50"/>
+      <c r="Q15" s="51"/>
       <c r="R15" s="18"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="24"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="38"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="45"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
@@ -1568,18 +1576,18 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
-      <c r="O16" s="43"/>
-      <c r="P16" s="43"/>
-      <c r="Q16" s="44"/>
+      <c r="O16" s="50"/>
+      <c r="P16" s="50"/>
+      <c r="Q16" s="51"/>
       <c r="R16" s="18"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="24"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="38"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="21"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -1588,18 +1596,18 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
-      <c r="O17" s="43"/>
-      <c r="P17" s="43"/>
-      <c r="Q17" s="44"/>
+      <c r="O17" s="29"/>
+      <c r="P17" s="30"/>
+      <c r="Q17" s="31"/>
       <c r="R17" s="18"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="38"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="21"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -1608,481 +1616,481 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
-      <c r="O18" s="43"/>
-      <c r="P18" s="43"/>
-      <c r="Q18" s="44"/>
+      <c r="O18" s="29"/>
+      <c r="P18" s="30"/>
+      <c r="Q18" s="31"/>
       <c r="R18" s="18"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="55" t="s">
+      <c r="A19" s="2"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="29"/>
+      <c r="P19" s="30"/>
+      <c r="Q19" s="31"/>
+      <c r="R19" s="18"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="30"/>
+      <c r="Q20" s="31"/>
+      <c r="R20" s="18"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="29"/>
+      <c r="P21" s="30"/>
+      <c r="Q21" s="31"/>
+      <c r="R21" s="18"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="29"/>
+      <c r="P22" s="30"/>
+      <c r="Q22" s="31"/>
+      <c r="R22" s="18"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="29"/>
+      <c r="P23" s="30"/>
+      <c r="Q23" s="31"/>
+      <c r="R23" s="18"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="29"/>
+      <c r="P24" s="30"/>
+      <c r="Q24" s="31"/>
+      <c r="R24" s="18"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="29"/>
+      <c r="P25" s="30"/>
+      <c r="Q25" s="31"/>
+      <c r="R25" s="18"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="32"/>
+      <c r="P26" s="33"/>
+      <c r="Q26" s="34"/>
+      <c r="R26" s="18"/>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="44"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="50"/>
+      <c r="P27" s="50"/>
+      <c r="Q27" s="51"/>
+      <c r="R27" s="18"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="56"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="45"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="50"/>
+      <c r="P28" s="50"/>
+      <c r="Q28" s="51"/>
+      <c r="R28" s="18"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A29" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="56"/>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="56"/>
-      <c r="J19" s="56"/>
-      <c r="K19" s="56"/>
-      <c r="L19" s="56"/>
-      <c r="M19" s="56"/>
-      <c r="N19" s="57"/>
-      <c r="O19" s="47" t="s">
+      <c r="B29" s="66"/>
+      <c r="C29" s="66"/>
+      <c r="D29" s="66"/>
+      <c r="E29" s="66"/>
+      <c r="F29" s="66"/>
+      <c r="G29" s="66"/>
+      <c r="H29" s="66"/>
+      <c r="I29" s="66"/>
+      <c r="J29" s="66"/>
+      <c r="K29" s="66"/>
+      <c r="L29" s="66"/>
+      <c r="M29" s="66"/>
+      <c r="N29" s="67"/>
+      <c r="O29" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="P19" s="47"/>
-      <c r="Q19" s="48"/>
-      <c r="R19" s="19"/>
-    </row>
-    <row r="20" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="58"/>
-      <c r="B20" s="59"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="59"/>
-      <c r="E20" s="59"/>
-      <c r="F20" s="59"/>
-      <c r="G20" s="59"/>
-      <c r="H20" s="59"/>
-      <c r="I20" s="59"/>
-      <c r="J20" s="59"/>
-      <c r="K20" s="59"/>
-      <c r="L20" s="59"/>
-      <c r="M20" s="59"/>
-      <c r="N20" s="60"/>
-      <c r="O20" s="49"/>
-      <c r="P20" s="49"/>
-      <c r="Q20" s="50"/>
-      <c r="R20" s="19"/>
-    </row>
-    <row r="21" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="20" t="s">
+      <c r="P29" s="57"/>
+      <c r="Q29" s="58"/>
+      <c r="R29" s="19"/>
+    </row>
+    <row r="30" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="68"/>
+      <c r="B30" s="69"/>
+      <c r="C30" s="69"/>
+      <c r="D30" s="69"/>
+      <c r="E30" s="69"/>
+      <c r="F30" s="69"/>
+      <c r="G30" s="69"/>
+      <c r="H30" s="69"/>
+      <c r="I30" s="69"/>
+      <c r="J30" s="69"/>
+      <c r="K30" s="69"/>
+      <c r="L30" s="69"/>
+      <c r="M30" s="69"/>
+      <c r="N30" s="70"/>
+      <c r="O30" s="59"/>
+      <c r="P30" s="59"/>
+      <c r="Q30" s="60"/>
+      <c r="R30" s="19"/>
+    </row>
+    <row r="31" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="13" t="s">
+      <c r="B31" s="20"/>
+      <c r="C31" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D31" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E21" s="52" t="s">
+      <c r="E31" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="F21" s="53"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="53"/>
-      <c r="I21" s="53"/>
-      <c r="J21" s="53"/>
-      <c r="K21" s="53"/>
-      <c r="L21" s="53"/>
-      <c r="M21" s="53"/>
-      <c r="N21" s="54"/>
-      <c r="O21" s="51"/>
-      <c r="P21" s="51"/>
-      <c r="Q21" s="34"/>
-      <c r="R21" s="19"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="8"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="61"/>
-      <c r="F22" s="61"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="35"/>
-      <c r="L22" s="36"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="41"/>
-      <c r="P22" s="41"/>
-      <c r="Q22" s="42"/>
-      <c r="R22" s="18"/>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23" s="4"/>
-      <c r="B23" s="24"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="62"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="37"/>
-      <c r="L23" s="38"/>
-      <c r="M23" s="21"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="43"/>
-      <c r="P23" s="43"/>
-      <c r="Q23" s="44"/>
-      <c r="R23" s="18"/>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="4"/>
-      <c r="B24" s="24"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
-      <c r="G24" s="62"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="37"/>
-      <c r="L24" s="38"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="3"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="43"/>
-      <c r="Q24" s="44"/>
-      <c r="R24" s="18"/>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="62"/>
-      <c r="G25" s="62"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="37"/>
-      <c r="L25" s="38"/>
-      <c r="M25" s="21"/>
-      <c r="N25" s="3"/>
-      <c r="O25" s="43"/>
-      <c r="P25" s="43"/>
-      <c r="Q25" s="44"/>
-      <c r="R25" s="18"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="4"/>
-      <c r="B26" s="24"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="62"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="37"/>
-      <c r="L26" s="38"/>
-      <c r="M26" s="21"/>
-      <c r="N26" s="3"/>
-      <c r="O26" s="43"/>
-      <c r="P26" s="43"/>
-      <c r="Q26" s="44"/>
-      <c r="R26" s="18"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27" s="4"/>
-      <c r="B27" s="24"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="62"/>
-      <c r="F27" s="62"/>
-      <c r="G27" s="62"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="37"/>
-      <c r="L27" s="38"/>
-      <c r="M27" s="21"/>
-      <c r="N27" s="3"/>
-      <c r="O27" s="43"/>
-      <c r="P27" s="43"/>
-      <c r="Q27" s="44"/>
-      <c r="R27" s="18"/>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="4"/>
-      <c r="B28" s="24"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="62"/>
-      <c r="F28" s="62"/>
-      <c r="G28" s="62"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="37"/>
-      <c r="L28" s="38"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="43"/>
-      <c r="P28" s="43"/>
-      <c r="Q28" s="44"/>
-      <c r="R28" s="18"/>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="10"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="62"/>
-      <c r="F29" s="62"/>
-      <c r="G29" s="62"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="37"/>
-      <c r="L29" s="38"/>
-      <c r="M29" s="21"/>
-      <c r="N29" s="7"/>
-      <c r="O29" s="43"/>
-      <c r="P29" s="43"/>
-      <c r="Q29" s="44"/>
-      <c r="R29" s="18"/>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="10"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="62"/>
-      <c r="F30" s="62"/>
-      <c r="G30" s="62"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="37"/>
-      <c r="L30" s="38"/>
-      <c r="M30" s="21"/>
-      <c r="N30" s="7"/>
-      <c r="O30" s="43"/>
-      <c r="P30" s="43"/>
-      <c r="Q30" s="44"/>
-      <c r="R30" s="18"/>
-    </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A31" s="10"/>
-      <c r="B31" s="26"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="62"/>
-      <c r="F31" s="62"/>
-      <c r="G31" s="62"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="37"/>
-      <c r="L31" s="38"/>
-      <c r="M31" s="21"/>
-      <c r="N31" s="7"/>
-      <c r="O31" s="43"/>
-      <c r="P31" s="43"/>
-      <c r="Q31" s="44"/>
-      <c r="R31" s="18"/>
+      <c r="F31" s="63"/>
+      <c r="G31" s="63"/>
+      <c r="H31" s="63"/>
+      <c r="I31" s="63"/>
+      <c r="J31" s="63"/>
+      <c r="K31" s="63"/>
+      <c r="L31" s="63"/>
+      <c r="M31" s="63"/>
+      <c r="N31" s="64"/>
+      <c r="O31" s="61"/>
+      <c r="P31" s="61"/>
+      <c r="Q31" s="41"/>
+      <c r="R31" s="19"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A32" s="7"/>
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="7"/>
-      <c r="K32" s="37"/>
-      <c r="L32" s="38"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="7"/>
-      <c r="O32" s="43"/>
-      <c r="P32" s="43"/>
-      <c r="Q32" s="43"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="71"/>
+      <c r="F32" s="71"/>
+      <c r="G32" s="71"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="9"/>
+      <c r="K32" s="42"/>
+      <c r="L32" s="43"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="6"/>
+      <c r="O32" s="48"/>
+      <c r="P32" s="48"/>
+      <c r="Q32" s="49"/>
       <c r="R32" s="18"/>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="43"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="37"/>
-      <c r="L33" s="38"/>
+      <c r="A33" s="4"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="72"/>
+      <c r="F33" s="72"/>
+      <c r="G33" s="72"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="44"/>
+      <c r="L33" s="45"/>
       <c r="M33" s="21"/>
-      <c r="N33" s="7"/>
-      <c r="O33" s="43"/>
-      <c r="P33" s="43"/>
-      <c r="Q33" s="43"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="50"/>
+      <c r="P33" s="50"/>
+      <c r="Q33" s="51"/>
       <c r="R33" s="18"/>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="37"/>
-      <c r="L34" s="38"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="72"/>
+      <c r="F34" s="72"/>
+      <c r="G34" s="72"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="44"/>
+      <c r="L34" s="45"/>
       <c r="M34" s="21"/>
-      <c r="N34" s="7"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="43"/>
-      <c r="Q34" s="43"/>
+      <c r="N34" s="3"/>
+      <c r="O34" s="50"/>
+      <c r="P34" s="50"/>
+      <c r="Q34" s="51"/>
       <c r="R34" s="18"/>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="63"/>
-      <c r="F35" s="64"/>
-      <c r="G35" s="65"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
-      <c r="J35" s="7"/>
-      <c r="K35" s="37"/>
-      <c r="L35" s="38"/>
+      <c r="A35" s="4"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="72"/>
+      <c r="F35" s="72"/>
+      <c r="G35" s="72"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="44"/>
+      <c r="L35" s="45"/>
       <c r="M35" s="21"/>
-      <c r="N35" s="7"/>
-      <c r="O35" s="43"/>
-      <c r="P35" s="43"/>
-      <c r="Q35" s="43"/>
+      <c r="N35" s="3"/>
+      <c r="O35" s="50"/>
+      <c r="P35" s="50"/>
+      <c r="Q35" s="51"/>
       <c r="R35" s="18"/>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="63"/>
-      <c r="F36" s="64"/>
-      <c r="G36" s="65"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="37"/>
-      <c r="L36" s="38"/>
+      <c r="A36" s="4"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="72"/>
+      <c r="F36" s="72"/>
+      <c r="G36" s="72"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="44"/>
+      <c r="L36" s="45"/>
       <c r="M36" s="21"/>
-      <c r="N36" s="7"/>
-      <c r="O36" s="43"/>
-      <c r="P36" s="43"/>
-      <c r="Q36" s="43"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="50"/>
+      <c r="P36" s="50"/>
+      <c r="Q36" s="51"/>
       <c r="R36" s="18"/>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="63"/>
-      <c r="F37" s="64"/>
-      <c r="G37" s="65"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="37"/>
-      <c r="L37" s="38"/>
+      <c r="A37" s="4"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="72"/>
+      <c r="F37" s="72"/>
+      <c r="G37" s="72"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="44"/>
+      <c r="L37" s="45"/>
       <c r="M37" s="21"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="43"/>
-      <c r="P37" s="43"/>
-      <c r="Q37" s="43"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="50"/>
+      <c r="P37" s="50"/>
+      <c r="Q37" s="51"/>
       <c r="R37" s="18"/>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="63"/>
-      <c r="F38" s="64"/>
-      <c r="G38" s="65"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="J38" s="7"/>
-      <c r="K38" s="37"/>
-      <c r="L38" s="38"/>
+      <c r="A38" s="4"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="72"/>
+      <c r="F38" s="72"/>
+      <c r="G38" s="72"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="44"/>
+      <c r="L38" s="45"/>
       <c r="M38" s="21"/>
-      <c r="N38" s="7"/>
-      <c r="O38" s="43"/>
-      <c r="P38" s="43"/>
-      <c r="Q38" s="43"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="50"/>
+      <c r="P38" s="50"/>
+      <c r="Q38" s="51"/>
       <c r="R38" s="18"/>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A39" s="7"/>
-      <c r="B39" s="7"/>
+      <c r="A39" s="10"/>
+      <c r="B39" s="26"/>
       <c r="C39" s="7"/>
       <c r="D39" s="7"/>
-      <c r="E39" s="63"/>
-      <c r="F39" s="64"/>
-      <c r="G39" s="65"/>
+      <c r="E39" s="72"/>
+      <c r="F39" s="72"/>
+      <c r="G39" s="72"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
-      <c r="J39" s="7"/>
-      <c r="K39" s="37"/>
-      <c r="L39" s="38"/>
+      <c r="J39" s="11"/>
+      <c r="K39" s="44"/>
+      <c r="L39" s="45"/>
       <c r="M39" s="21"/>
       <c r="N39" s="7"/>
-      <c r="O39" s="43"/>
-      <c r="P39" s="43"/>
-      <c r="Q39" s="43"/>
+      <c r="O39" s="50"/>
+      <c r="P39" s="50"/>
+      <c r="Q39" s="51"/>
       <c r="R39" s="18"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A40" s="7"/>
-      <c r="B40" s="7"/>
+      <c r="A40" s="10"/>
+      <c r="B40" s="26"/>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
-      <c r="E40" s="63"/>
-      <c r="F40" s="64"/>
-      <c r="G40" s="65"/>
+      <c r="E40" s="72"/>
+      <c r="F40" s="72"/>
+      <c r="G40" s="72"/>
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
-      <c r="J40" s="7"/>
-      <c r="K40" s="37"/>
-      <c r="L40" s="38"/>
+      <c r="J40" s="11"/>
+      <c r="K40" s="44"/>
+      <c r="L40" s="45"/>
       <c r="M40" s="21"/>
       <c r="N40" s="7"/>
-      <c r="O40" s="43"/>
-      <c r="P40" s="43"/>
-      <c r="Q40" s="43"/>
+      <c r="O40" s="50"/>
+      <c r="P40" s="50"/>
+      <c r="Q40" s="51"/>
       <c r="R40" s="18"/>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
+      <c r="A41" s="10"/>
+      <c r="B41" s="26"/>
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
-      <c r="E41" s="63"/>
-      <c r="F41" s="64"/>
-      <c r="G41" s="65"/>
+      <c r="E41" s="72"/>
+      <c r="F41" s="72"/>
+      <c r="G41" s="72"/>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
-      <c r="J41" s="7"/>
-      <c r="K41" s="37"/>
-      <c r="L41" s="38"/>
+      <c r="J41" s="11"/>
+      <c r="K41" s="44"/>
+      <c r="L41" s="45"/>
       <c r="M41" s="21"/>
       <c r="N41" s="7"/>
-      <c r="O41" s="43"/>
-      <c r="P41" s="43"/>
-      <c r="Q41" s="43"/>
+      <c r="O41" s="50"/>
+      <c r="P41" s="50"/>
+      <c r="Q41" s="51"/>
       <c r="R41" s="18"/>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
@@ -2090,19 +2098,19 @@
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
-      <c r="E42" s="63"/>
-      <c r="F42" s="64"/>
-      <c r="G42" s="65"/>
+      <c r="E42" s="50"/>
+      <c r="F42" s="50"/>
+      <c r="G42" s="50"/>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
       <c r="J42" s="7"/>
-      <c r="K42" s="37"/>
-      <c r="L42" s="38"/>
+      <c r="K42" s="44"/>
+      <c r="L42" s="45"/>
       <c r="M42" s="21"/>
       <c r="N42" s="7"/>
-      <c r="O42" s="43"/>
-      <c r="P42" s="43"/>
-      <c r="Q42" s="43"/>
+      <c r="O42" s="50"/>
+      <c r="P42" s="50"/>
+      <c r="Q42" s="50"/>
       <c r="R42" s="18"/>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
@@ -2110,19 +2118,19 @@
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
       <c r="D43" s="7"/>
-      <c r="E43" s="63"/>
-      <c r="F43" s="64"/>
-      <c r="G43" s="65"/>
+      <c r="E43" s="50"/>
+      <c r="F43" s="50"/>
+      <c r="G43" s="50"/>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
       <c r="J43" s="7"/>
-      <c r="K43" s="37"/>
-      <c r="L43" s="38"/>
+      <c r="K43" s="44"/>
+      <c r="L43" s="45"/>
       <c r="M43" s="21"/>
       <c r="N43" s="7"/>
-      <c r="O43" s="43"/>
-      <c r="P43" s="43"/>
-      <c r="Q43" s="43"/>
+      <c r="O43" s="50"/>
+      <c r="P43" s="50"/>
+      <c r="Q43" s="50"/>
       <c r="R43" s="18"/>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
@@ -2130,19 +2138,19 @@
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
-      <c r="E44" s="63"/>
-      <c r="F44" s="64"/>
-      <c r="G44" s="65"/>
+      <c r="E44" s="50"/>
+      <c r="F44" s="50"/>
+      <c r="G44" s="50"/>
       <c r="H44" s="7"/>
       <c r="I44" s="7"/>
       <c r="J44" s="7"/>
-      <c r="K44" s="37"/>
-      <c r="L44" s="38"/>
+      <c r="K44" s="44"/>
+      <c r="L44" s="45"/>
       <c r="M44" s="21"/>
       <c r="N44" s="7"/>
-      <c r="O44" s="43"/>
-      <c r="P44" s="43"/>
-      <c r="Q44" s="43"/>
+      <c r="O44" s="50"/>
+      <c r="P44" s="50"/>
+      <c r="Q44" s="50"/>
       <c r="R44" s="18"/>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
@@ -2150,19 +2158,19 @@
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
-      <c r="E45" s="63"/>
-      <c r="F45" s="64"/>
-      <c r="G45" s="65"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="73"/>
       <c r="H45" s="7"/>
       <c r="I45" s="7"/>
       <c r="J45" s="7"/>
-      <c r="K45" s="37"/>
-      <c r="L45" s="38"/>
+      <c r="K45" s="44"/>
+      <c r="L45" s="45"/>
       <c r="M45" s="21"/>
       <c r="N45" s="7"/>
-      <c r="O45" s="43"/>
-      <c r="P45" s="43"/>
-      <c r="Q45" s="43"/>
+      <c r="O45" s="50"/>
+      <c r="P45" s="50"/>
+      <c r="Q45" s="50"/>
       <c r="R45" s="18"/>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
@@ -2170,19 +2178,19 @@
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
-      <c r="E46" s="63"/>
-      <c r="F46" s="64"/>
-      <c r="G46" s="65"/>
+      <c r="E46" s="32"/>
+      <c r="F46" s="33"/>
+      <c r="G46" s="73"/>
       <c r="H46" s="7"/>
       <c r="I46" s="7"/>
       <c r="J46" s="7"/>
-      <c r="K46" s="37"/>
-      <c r="L46" s="38"/>
+      <c r="K46" s="44"/>
+      <c r="L46" s="45"/>
       <c r="M46" s="21"/>
       <c r="N46" s="7"/>
-      <c r="O46" s="43"/>
-      <c r="P46" s="43"/>
-      <c r="Q46" s="43"/>
+      <c r="O46" s="50"/>
+      <c r="P46" s="50"/>
+      <c r="Q46" s="50"/>
       <c r="R46" s="18"/>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
@@ -2190,19 +2198,19 @@
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="63"/>
-      <c r="F47" s="64"/>
-      <c r="G47" s="65"/>
+      <c r="E47" s="32"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="73"/>
       <c r="H47" s="7"/>
       <c r="I47" s="7"/>
       <c r="J47" s="7"/>
-      <c r="K47" s="37"/>
-      <c r="L47" s="38"/>
+      <c r="K47" s="44"/>
+      <c r="L47" s="45"/>
       <c r="M47" s="21"/>
       <c r="N47" s="7"/>
-      <c r="O47" s="43"/>
-      <c r="P47" s="43"/>
-      <c r="Q47" s="43"/>
+      <c r="O47" s="50"/>
+      <c r="P47" s="50"/>
+      <c r="Q47" s="50"/>
       <c r="R47" s="18"/>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
@@ -2210,19 +2218,19 @@
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
-      <c r="E48" s="63"/>
-      <c r="F48" s="64"/>
-      <c r="G48" s="65"/>
+      <c r="E48" s="32"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="73"/>
       <c r="H48" s="7"/>
       <c r="I48" s="7"/>
       <c r="J48" s="7"/>
-      <c r="K48" s="37"/>
-      <c r="L48" s="38"/>
+      <c r="K48" s="44"/>
+      <c r="L48" s="45"/>
       <c r="M48" s="21"/>
       <c r="N48" s="7"/>
-      <c r="O48" s="43"/>
-      <c r="P48" s="43"/>
-      <c r="Q48" s="43"/>
+      <c r="O48" s="50"/>
+      <c r="P48" s="50"/>
+      <c r="Q48" s="50"/>
       <c r="R48" s="18"/>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
@@ -2230,19 +2238,19 @@
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
-      <c r="E49" s="63"/>
-      <c r="F49" s="64"/>
-      <c r="G49" s="65"/>
+      <c r="E49" s="32"/>
+      <c r="F49" s="33"/>
+      <c r="G49" s="73"/>
       <c r="H49" s="7"/>
       <c r="I49" s="7"/>
       <c r="J49" s="7"/>
-      <c r="K49" s="37"/>
-      <c r="L49" s="38"/>
+      <c r="K49" s="44"/>
+      <c r="L49" s="45"/>
       <c r="M49" s="21"/>
       <c r="N49" s="7"/>
-      <c r="O49" s="43"/>
-      <c r="P49" s="43"/>
-      <c r="Q49" s="43"/>
+      <c r="O49" s="50"/>
+      <c r="P49" s="50"/>
+      <c r="Q49" s="50"/>
       <c r="R49" s="18"/>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
@@ -2250,28 +2258,238 @@
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
       <c r="D50" s="7"/>
-      <c r="E50" s="63"/>
-      <c r="F50" s="64"/>
-      <c r="G50" s="65"/>
+      <c r="E50" s="32"/>
+      <c r="F50" s="33"/>
+      <c r="G50" s="73"/>
       <c r="H50" s="7"/>
       <c r="I50" s="7"/>
       <c r="J50" s="7"/>
-      <c r="K50" s="37"/>
-      <c r="L50" s="38"/>
+      <c r="K50" s="44"/>
+      <c r="L50" s="45"/>
       <c r="M50" s="21"/>
       <c r="N50" s="7"/>
-      <c r="O50" s="43"/>
-      <c r="P50" s="43"/>
-      <c r="Q50" s="43"/>
+      <c r="O50" s="50"/>
+      <c r="P50" s="50"/>
+      <c r="Q50" s="50"/>
       <c r="R50" s="18"/>
     </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="32"/>
+      <c r="F51" s="33"/>
+      <c r="G51" s="73"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="7"/>
+      <c r="J51" s="7"/>
+      <c r="K51" s="44"/>
+      <c r="L51" s="45"/>
+      <c r="M51" s="21"/>
+      <c r="N51" s="7"/>
+      <c r="O51" s="50"/>
+      <c r="P51" s="50"/>
+      <c r="Q51" s="50"/>
+      <c r="R51" s="18"/>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A52" s="7"/>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="32"/>
+      <c r="F52" s="33"/>
+      <c r="G52" s="73"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="7"/>
+      <c r="J52" s="7"/>
+      <c r="K52" s="44"/>
+      <c r="L52" s="45"/>
+      <c r="M52" s="21"/>
+      <c r="N52" s="7"/>
+      <c r="O52" s="50"/>
+      <c r="P52" s="50"/>
+      <c r="Q52" s="50"/>
+      <c r="R52" s="18"/>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="32"/>
+      <c r="F53" s="33"/>
+      <c r="G53" s="73"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+      <c r="J53" s="7"/>
+      <c r="K53" s="44"/>
+      <c r="L53" s="45"/>
+      <c r="M53" s="21"/>
+      <c r="N53" s="7"/>
+      <c r="O53" s="50"/>
+      <c r="P53" s="50"/>
+      <c r="Q53" s="50"/>
+      <c r="R53" s="18"/>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A54" s="7"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="32"/>
+      <c r="F54" s="33"/>
+      <c r="G54" s="73"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+      <c r="J54" s="7"/>
+      <c r="K54" s="44"/>
+      <c r="L54" s="45"/>
+      <c r="M54" s="21"/>
+      <c r="N54" s="7"/>
+      <c r="O54" s="50"/>
+      <c r="P54" s="50"/>
+      <c r="Q54" s="50"/>
+      <c r="R54" s="18"/>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A55" s="7"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="32"/>
+      <c r="F55" s="33"/>
+      <c r="G55" s="73"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+      <c r="K55" s="44"/>
+      <c r="L55" s="45"/>
+      <c r="M55" s="21"/>
+      <c r="N55" s="7"/>
+      <c r="O55" s="50"/>
+      <c r="P55" s="50"/>
+      <c r="Q55" s="50"/>
+      <c r="R55" s="18"/>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A56" s="7"/>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="32"/>
+      <c r="F56" s="33"/>
+      <c r="G56" s="73"/>
+      <c r="H56" s="7"/>
+      <c r="I56" s="7"/>
+      <c r="J56" s="7"/>
+      <c r="K56" s="44"/>
+      <c r="L56" s="45"/>
+      <c r="M56" s="21"/>
+      <c r="N56" s="7"/>
+      <c r="O56" s="50"/>
+      <c r="P56" s="50"/>
+      <c r="Q56" s="50"/>
+      <c r="R56" s="18"/>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A57" s="7"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="32"/>
+      <c r="F57" s="33"/>
+      <c r="G57" s="73"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="44"/>
+      <c r="L57" s="45"/>
+      <c r="M57" s="21"/>
+      <c r="N57" s="7"/>
+      <c r="O57" s="50"/>
+      <c r="P57" s="50"/>
+      <c r="Q57" s="50"/>
+      <c r="R57" s="18"/>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A58" s="7"/>
+      <c r="B58" s="7"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
+      <c r="E58" s="32"/>
+      <c r="F58" s="33"/>
+      <c r="G58" s="73"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+      <c r="J58" s="7"/>
+      <c r="K58" s="44"/>
+      <c r="L58" s="45"/>
+      <c r="M58" s="21"/>
+      <c r="N58" s="7"/>
+      <c r="O58" s="50"/>
+      <c r="P58" s="50"/>
+      <c r="Q58" s="50"/>
+      <c r="R58" s="18"/>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A59" s="7"/>
+      <c r="B59" s="7"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="32"/>
+      <c r="F59" s="33"/>
+      <c r="G59" s="73"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+      <c r="K59" s="44"/>
+      <c r="L59" s="45"/>
+      <c r="M59" s="21"/>
+      <c r="N59" s="7"/>
+      <c r="O59" s="50"/>
+      <c r="P59" s="50"/>
+      <c r="Q59" s="50"/>
+      <c r="R59" s="18"/>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A60" s="7"/>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="7"/>
+      <c r="E60" s="32"/>
+      <c r="F60" s="33"/>
+      <c r="G60" s="73"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+      <c r="J60" s="7"/>
+      <c r="K60" s="44"/>
+      <c r="L60" s="45"/>
+      <c r="M60" s="21"/>
+      <c r="N60" s="7"/>
+      <c r="O60" s="50"/>
+      <c r="P60" s="50"/>
+      <c r="Q60" s="50"/>
+      <c r="R60" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="142">
+  <mergeCells count="143">
+    <mergeCell ref="K57:L57"/>
+    <mergeCell ref="K58:L58"/>
+    <mergeCell ref="K59:L59"/>
+    <mergeCell ref="K60:L60"/>
+    <mergeCell ref="K46:L46"/>
     <mergeCell ref="K47:L47"/>
     <mergeCell ref="K48:L48"/>
     <mergeCell ref="K49:L49"/>
     <mergeCell ref="K50:L50"/>
-    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="K51:L51"/>
+    <mergeCell ref="K52:L52"/>
+    <mergeCell ref="K53:L53"/>
+    <mergeCell ref="K54:L54"/>
+    <mergeCell ref="K55:L55"/>
+    <mergeCell ref="K56:L56"/>
     <mergeCell ref="K37:L37"/>
     <mergeCell ref="K38:L38"/>
     <mergeCell ref="K39:L39"/>
@@ -2280,86 +2498,76 @@
     <mergeCell ref="K42:L42"/>
     <mergeCell ref="K43:L43"/>
     <mergeCell ref="K44:L44"/>
-    <mergeCell ref="K45:L45"/>
-    <mergeCell ref="K46:L46"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="O56:Q56"/>
+    <mergeCell ref="O57:Q57"/>
+    <mergeCell ref="O58:Q58"/>
+    <mergeCell ref="O59:Q59"/>
+    <mergeCell ref="O60:Q60"/>
+    <mergeCell ref="O43:Q43"/>
+    <mergeCell ref="O44:Q44"/>
+    <mergeCell ref="O45:Q45"/>
     <mergeCell ref="O46:Q46"/>
     <mergeCell ref="O47:Q47"/>
     <mergeCell ref="O48:Q48"/>
     <mergeCell ref="O49:Q49"/>
     <mergeCell ref="O50:Q50"/>
-    <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="O34:Q34"/>
-    <mergeCell ref="O35:Q35"/>
-    <mergeCell ref="O36:Q36"/>
-    <mergeCell ref="O37:Q37"/>
+    <mergeCell ref="O51:Q51"/>
+    <mergeCell ref="O52:Q52"/>
+    <mergeCell ref="O53:Q53"/>
+    <mergeCell ref="O54:Q54"/>
+    <mergeCell ref="O55:Q55"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="E60:G60"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="E54:G54"/>
+    <mergeCell ref="E55:G55"/>
+    <mergeCell ref="E56:G56"/>
+    <mergeCell ref="E38:G38"/>
     <mergeCell ref="O38:Q38"/>
     <mergeCell ref="O39:Q39"/>
     <mergeCell ref="O40:Q40"/>
-    <mergeCell ref="O41:Q41"/>
-    <mergeCell ref="O42:Q42"/>
-    <mergeCell ref="O43:Q43"/>
-    <mergeCell ref="O44:Q44"/>
-    <mergeCell ref="O45:Q45"/>
-    <mergeCell ref="E47:G47"/>
     <mergeCell ref="E48:G48"/>
     <mergeCell ref="E49:G49"/>
     <mergeCell ref="E50:G50"/>
-    <mergeCell ref="E41:G41"/>
     <mergeCell ref="E42:G42"/>
     <mergeCell ref="E43:G43"/>
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="E45:G45"/>
-    <mergeCell ref="E46:G46"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="O30:Q30"/>
-    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="O41:Q41"/>
+    <mergeCell ref="O42:Q42"/>
+    <mergeCell ref="K45:L45"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="E40:G40"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="E46:G46"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="O29:Q31"/>
+    <mergeCell ref="O37:Q37"/>
+    <mergeCell ref="O35:Q35"/>
+    <mergeCell ref="O36:Q36"/>
+    <mergeCell ref="E31:N31"/>
+    <mergeCell ref="A29:N30"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="O28:Q28"/>
+    <mergeCell ref="O12:Q12"/>
     <mergeCell ref="E32:G32"/>
-    <mergeCell ref="E33:G33"/>
-    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="O32:Q32"/>
     <mergeCell ref="E35:G35"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="O32:Q32"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="E31:G31"/>
     <mergeCell ref="E36:G36"/>
     <mergeCell ref="E37:G37"/>
-    <mergeCell ref="O19:Q21"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="O25:Q25"/>
-    <mergeCell ref="O26:Q26"/>
-    <mergeCell ref="E21:N21"/>
-    <mergeCell ref="A19:N20"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="O18:Q18"/>
-    <mergeCell ref="O12:Q12"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="O22:Q22"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="O24:Q24"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="E33:G33"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="O34:Q34"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="E34:G34"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="O13:Q13"/>
     <mergeCell ref="O14:Q14"/>
@@ -2370,32 +2578,23 @@
     <mergeCell ref="O9:Q9"/>
     <mergeCell ref="O10:Q10"/>
     <mergeCell ref="O11:Q11"/>
+    <mergeCell ref="C8:D8"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="O26:Q26"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="J2:K2"/>
     <mergeCell ref="M2:N2"/>
@@ -2409,6 +2608,16 @@
     <mergeCell ref="O5:Q5"/>
     <mergeCell ref="O6:Q6"/>
     <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <printOptions headings="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Refinamento das formatações do Laudo
</commit_message>
<xml_diff>
--- a/modelos/apontamento_manha.xlsx
+++ b/modelos/apontamento_manha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{5CF2130B-03D7-4201-A06E-E31242A6816B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{863DF637-E67F-4125-AFAC-C3AD3DDD928C}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{5CF2130B-03D7-4201-A06E-E31242A6816B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7C1BF54-FA7C-4049-9B1F-50D2324E7496}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{18B97131-922C-4537-B241-F72155183AFA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -96,6 +96,15 @@
   </si>
   <si>
     <t>APONTAMENTO DE PRODUÇÃO - NOITE</t>
+  </si>
+  <si>
+    <t>META</t>
+  </si>
+  <si>
+    <t>DATA</t>
+  </si>
+  <si>
+    <t>OPERADOR</t>
   </si>
 </sst>
 </file>
@@ -178,7 +187,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="39">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -466,30 +475,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -623,19 +608,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="medium">
         <color indexed="64"/>
@@ -652,7 +624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -669,145 +641,124 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -840,6 +791,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -868,8 +828,8 @@
       <xdr:rowOff>109536</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1185863</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>490537</xdr:rowOff>
     </xdr:to>
@@ -909,6 +869,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1231,65 +1195,77 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R60"/>
+  <dimension ref="A1:S60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="4" width="11" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
     <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="28.5703125" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="11.5703125" customWidth="1"/>
-    <col min="10" max="11" width="14.140625" customWidth="1"/>
-    <col min="12" max="12" width="30.5703125" customWidth="1"/>
-    <col min="13" max="13" width="16.140625" customWidth="1"/>
-    <col min="14" max="14" width="19.7109375" customWidth="1"/>
-    <col min="16" max="16" width="8" customWidth="1"/>
-    <col min="17" max="17" width="10.28515625" customWidth="1"/>
-    <col min="18" max="18" width="5.28515625" customWidth="1"/>
+    <col min="10" max="12" width="14.28515625" customWidth="1"/>
+    <col min="13" max="13" width="21.42578125" customWidth="1"/>
+    <col min="14" max="14" width="16.140625" customWidth="1"/>
+    <col min="15" max="15" width="19.7109375" customWidth="1"/>
+    <col min="16" max="16" width="13.5703125" customWidth="1"/>
+    <col min="17" max="17" width="8" customWidth="1"/>
+    <col min="18" max="18" width="10.28515625" customWidth="1"/>
+    <col min="19" max="19" width="5.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:18" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
+    <row r="2" spans="1:19" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="39"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="38"/>
-      <c r="N2" s="39"/>
-      <c r="O2" s="52"/>
-      <c r="P2" s="53"/>
-      <c r="Q2" s="54"/>
-      <c r="R2" s="17"/>
-    </row>
-    <row r="3" spans="1:18" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="69" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="67"/>
+      <c r="L2" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" s="67"/>
+      <c r="N2" s="69" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="67"/>
+      <c r="P2" s="69" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q2" s="68"/>
+      <c r="R2" s="68"/>
+      <c r="S2" s="17"/>
+    </row>
+    <row r="3" spans="1:19" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="41"/>
-      <c r="E3" s="40" t="s">
+      <c r="D3" s="37"/>
+      <c r="E3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="41"/>
+      <c r="F3" s="37"/>
       <c r="G3" s="14" t="s">
         <v>2</v>
       </c>
@@ -1302,32 +1278,33 @@
       <c r="J3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="15" t="s">
+      <c r="K3" s="15"/>
+      <c r="L3" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="M3" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="16" t="s">
+      <c r="N3" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="16" t="s">
+      <c r="O3" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="O3" s="46" t="s">
+      <c r="P3" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="P3" s="46"/>
-      <c r="Q3" s="47"/>
-      <c r="R3" s="19"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q3" s="42"/>
+      <c r="R3" s="43"/>
+      <c r="S3" s="19"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="12"/>
       <c r="B4" s="23"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="43"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="39"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
@@ -1336,18 +1313,19 @@
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
-      <c r="O4" s="48"/>
-      <c r="P4" s="48"/>
-      <c r="Q4" s="49"/>
-      <c r="R4" s="18"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O4" s="6"/>
+      <c r="P4" s="44"/>
+      <c r="Q4" s="44"/>
+      <c r="R4" s="45"/>
+      <c r="S4" s="18"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="24"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="45"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="41"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1356,18 +1334,19 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
-      <c r="O5" s="50"/>
-      <c r="P5" s="50"/>
-      <c r="Q5" s="51"/>
-      <c r="R5" s="18"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O5" s="3"/>
+      <c r="P5" s="46"/>
+      <c r="Q5" s="46"/>
+      <c r="R5" s="47"/>
+      <c r="S5" s="18"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="24"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="45"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="41"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -1376,18 +1355,19 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
-      <c r="O6" s="50"/>
-      <c r="P6" s="50"/>
-      <c r="Q6" s="51"/>
-      <c r="R6" s="18"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O6" s="3"/>
+      <c r="P6" s="46"/>
+      <c r="Q6" s="46"/>
+      <c r="R6" s="47"/>
+      <c r="S6" s="18"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="24"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="45"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="41"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -1396,18 +1376,19 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
-      <c r="O7" s="50"/>
-      <c r="P7" s="50"/>
-      <c r="Q7" s="51"/>
-      <c r="R7" s="18"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O7" s="3"/>
+      <c r="P7" s="46"/>
+      <c r="Q7" s="46"/>
+      <c r="R7" s="47"/>
+      <c r="S7" s="18"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="24"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="45"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="41"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -1416,18 +1397,19 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
-      <c r="O8" s="50"/>
-      <c r="P8" s="50"/>
-      <c r="Q8" s="51"/>
-      <c r="R8" s="18"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O8" s="3"/>
+      <c r="P8" s="46"/>
+      <c r="Q8" s="46"/>
+      <c r="R8" s="47"/>
+      <c r="S8" s="18"/>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="24"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="45"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="41"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -1436,18 +1418,19 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
-      <c r="O9" s="50"/>
-      <c r="P9" s="50"/>
-      <c r="Q9" s="51"/>
-      <c r="R9" s="18"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O9" s="3"/>
+      <c r="P9" s="46"/>
+      <c r="Q9" s="46"/>
+      <c r="R9" s="47"/>
+      <c r="S9" s="18"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="24"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="45"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="41"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -1456,18 +1439,19 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
-      <c r="O10" s="50"/>
-      <c r="P10" s="50"/>
-      <c r="Q10" s="51"/>
-      <c r="R10" s="18"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O10" s="3"/>
+      <c r="P10" s="46"/>
+      <c r="Q10" s="46"/>
+      <c r="R10" s="47"/>
+      <c r="S10" s="18"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="24"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="45"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="41"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -1476,18 +1460,19 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
-      <c r="O11" s="50"/>
-      <c r="P11" s="50"/>
-      <c r="Q11" s="51"/>
-      <c r="R11" s="18"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O11" s="3"/>
+      <c r="P11" s="46"/>
+      <c r="Q11" s="46"/>
+      <c r="R11" s="47"/>
+      <c r="S11" s="18"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="24"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="45"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="41"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
@@ -1496,18 +1481,19 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
-      <c r="O12" s="50"/>
-      <c r="P12" s="50"/>
-      <c r="Q12" s="51"/>
-      <c r="R12" s="18"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O12" s="3"/>
+      <c r="P12" s="46"/>
+      <c r="Q12" s="46"/>
+      <c r="R12" s="47"/>
+      <c r="S12" s="18"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="24"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="45"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="41"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -1516,18 +1502,19 @@
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
-      <c r="O13" s="50"/>
-      <c r="P13" s="50"/>
-      <c r="Q13" s="51"/>
-      <c r="R13" s="18"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O13" s="3"/>
+      <c r="P13" s="46"/>
+      <c r="Q13" s="46"/>
+      <c r="R13" s="47"/>
+      <c r="S13" s="18"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="24"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="45"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="41"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -1536,18 +1523,19 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
-      <c r="O14" s="50"/>
-      <c r="P14" s="50"/>
-      <c r="Q14" s="51"/>
-      <c r="R14" s="18"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O14" s="3"/>
+      <c r="P14" s="46"/>
+      <c r="Q14" s="46"/>
+      <c r="R14" s="47"/>
+      <c r="S14" s="18"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="24"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="45"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="41"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -1556,18 +1544,19 @@
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
-      <c r="O15" s="50"/>
-      <c r="P15" s="50"/>
-      <c r="Q15" s="51"/>
-      <c r="R15" s="18"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O15" s="3"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="47"/>
+      <c r="S15" s="18"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="24"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="44"/>
-      <c r="F16" s="45"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="41"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
@@ -1576,17 +1565,18 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
-      <c r="O16" s="50"/>
-      <c r="P16" s="50"/>
-      <c r="Q16" s="51"/>
-      <c r="R16" s="18"/>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O16" s="3"/>
+      <c r="P16" s="46"/>
+      <c r="Q16" s="46"/>
+      <c r="R16" s="47"/>
+      <c r="S16" s="18"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="24"/>
-      <c r="C17" s="28"/>
+      <c r="C17" s="27"/>
       <c r="D17" s="21"/>
-      <c r="E17" s="28"/>
+      <c r="E17" s="27"/>
       <c r="F17" s="21"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -1596,17 +1586,18 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
-      <c r="O17" s="29"/>
-      <c r="P17" s="30"/>
-      <c r="Q17" s="31"/>
-      <c r="R17" s="18"/>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O17" s="3"/>
+      <c r="P17" s="28"/>
+      <c r="Q17" s="29"/>
+      <c r="R17" s="30"/>
+      <c r="S17" s="18"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="24"/>
-      <c r="C18" s="28"/>
+      <c r="C18" s="27"/>
       <c r="D18" s="21"/>
-      <c r="E18" s="28"/>
+      <c r="E18" s="27"/>
       <c r="F18" s="21"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
@@ -1616,17 +1607,18 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
-      <c r="O18" s="29"/>
-      <c r="P18" s="30"/>
-      <c r="Q18" s="31"/>
-      <c r="R18" s="18"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O18" s="3"/>
+      <c r="P18" s="28"/>
+      <c r="Q18" s="29"/>
+      <c r="R18" s="30"/>
+      <c r="S18" s="18"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="24"/>
-      <c r="C19" s="28"/>
+      <c r="C19" s="27"/>
       <c r="D19" s="21"/>
-      <c r="E19" s="28"/>
+      <c r="E19" s="27"/>
       <c r="F19" s="21"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
@@ -1636,17 +1628,18 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
-      <c r="O19" s="29"/>
-      <c r="P19" s="30"/>
-      <c r="Q19" s="31"/>
-      <c r="R19" s="18"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O19" s="3"/>
+      <c r="P19" s="28"/>
+      <c r="Q19" s="29"/>
+      <c r="R19" s="30"/>
+      <c r="S19" s="18"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="24"/>
-      <c r="C20" s="28"/>
+      <c r="C20" s="27"/>
       <c r="D20" s="21"/>
-      <c r="E20" s="28"/>
+      <c r="E20" s="27"/>
       <c r="F20" s="21"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
@@ -1656,17 +1649,18 @@
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
-      <c r="O20" s="29"/>
-      <c r="P20" s="30"/>
-      <c r="Q20" s="31"/>
-      <c r="R20" s="18"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O20" s="3"/>
+      <c r="P20" s="28"/>
+      <c r="Q20" s="29"/>
+      <c r="R20" s="30"/>
+      <c r="S20" s="18"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="24"/>
-      <c r="C21" s="28"/>
+      <c r="C21" s="27"/>
       <c r="D21" s="21"/>
-      <c r="E21" s="28"/>
+      <c r="E21" s="27"/>
       <c r="F21" s="21"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
@@ -1676,17 +1670,18 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
-      <c r="O21" s="29"/>
-      <c r="P21" s="30"/>
-      <c r="Q21" s="31"/>
-      <c r="R21" s="18"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O21" s="3"/>
+      <c r="P21" s="28"/>
+      <c r="Q21" s="29"/>
+      <c r="R21" s="30"/>
+      <c r="S21" s="18"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="24"/>
-      <c r="C22" s="28"/>
+      <c r="C22" s="27"/>
       <c r="D22" s="21"/>
-      <c r="E22" s="28"/>
+      <c r="E22" s="27"/>
       <c r="F22" s="21"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
@@ -1696,17 +1691,18 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
-      <c r="O22" s="29"/>
-      <c r="P22" s="30"/>
-      <c r="Q22" s="31"/>
-      <c r="R22" s="18"/>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O22" s="3"/>
+      <c r="P22" s="28"/>
+      <c r="Q22" s="29"/>
+      <c r="R22" s="30"/>
+      <c r="S22" s="18"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="24"/>
-      <c r="C23" s="28"/>
+      <c r="C23" s="27"/>
       <c r="D23" s="21"/>
-      <c r="E23" s="28"/>
+      <c r="E23" s="27"/>
       <c r="F23" s="21"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
@@ -1716,17 +1712,18 @@
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
-      <c r="O23" s="29"/>
-      <c r="P23" s="30"/>
-      <c r="Q23" s="31"/>
-      <c r="R23" s="18"/>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O23" s="3"/>
+      <c r="P23" s="28"/>
+      <c r="Q23" s="29"/>
+      <c r="R23" s="30"/>
+      <c r="S23" s="18"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="24"/>
-      <c r="C24" s="28"/>
+      <c r="C24" s="27"/>
       <c r="D24" s="21"/>
-      <c r="E24" s="28"/>
+      <c r="E24" s="27"/>
       <c r="F24" s="21"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
@@ -1736,17 +1733,18 @@
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
-      <c r="O24" s="29"/>
-      <c r="P24" s="30"/>
-      <c r="Q24" s="31"/>
-      <c r="R24" s="18"/>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O24" s="3"/>
+      <c r="P24" s="28"/>
+      <c r="Q24" s="29"/>
+      <c r="R24" s="30"/>
+      <c r="S24" s="18"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="24"/>
-      <c r="C25" s="28"/>
+      <c r="C25" s="27"/>
       <c r="D25" s="21"/>
-      <c r="E25" s="28"/>
+      <c r="E25" s="27"/>
       <c r="F25" s="21"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
@@ -1756,17 +1754,18 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
-      <c r="O25" s="29"/>
-      <c r="P25" s="30"/>
-      <c r="Q25" s="31"/>
-      <c r="R25" s="18"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O25" s="3"/>
+      <c r="P25" s="28"/>
+      <c r="Q25" s="29"/>
+      <c r="R25" s="30"/>
+      <c r="S25" s="18"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="24"/>
-      <c r="C26" s="28"/>
+      <c r="C26" s="27"/>
       <c r="D26" s="21"/>
-      <c r="E26" s="28"/>
+      <c r="E26" s="27"/>
       <c r="F26" s="21"/>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
@@ -1776,18 +1775,19 @@
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
-      <c r="O26" s="32"/>
-      <c r="P26" s="33"/>
-      <c r="Q26" s="34"/>
-      <c r="R26" s="18"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O26" s="3"/>
+      <c r="P26" s="31"/>
+      <c r="Q26" s="32"/>
+      <c r="R26" s="33"/>
+      <c r="S26" s="18"/>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="24"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="45"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="45"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="41"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
@@ -1796,18 +1796,19 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
-      <c r="O27" s="50"/>
-      <c r="P27" s="50"/>
-      <c r="Q27" s="51"/>
-      <c r="R27" s="18"/>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O27" s="3"/>
+      <c r="P27" s="46"/>
+      <c r="Q27" s="46"/>
+      <c r="R27" s="47"/>
+      <c r="S27" s="18"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="25"/>
-      <c r="C28" s="55"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="44"/>
-      <c r="F28" s="45"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="41"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -1816,56 +1817,59 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
       <c r="N28" s="3"/>
-      <c r="O28" s="50"/>
-      <c r="P28" s="50"/>
-      <c r="Q28" s="51"/>
-      <c r="R28" s="18"/>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="65" t="s">
+      <c r="O28" s="3"/>
+      <c r="P28" s="46"/>
+      <c r="Q28" s="46"/>
+      <c r="R28" s="47"/>
+      <c r="S28" s="18"/>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A29" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="66"/>
-      <c r="C29" s="66"/>
-      <c r="D29" s="66"/>
-      <c r="E29" s="66"/>
-      <c r="F29" s="66"/>
-      <c r="G29" s="66"/>
-      <c r="H29" s="66"/>
-      <c r="I29" s="66"/>
-      <c r="J29" s="66"/>
-      <c r="K29" s="66"/>
-      <c r="L29" s="66"/>
-      <c r="M29" s="66"/>
-      <c r="N29" s="67"/>
-      <c r="O29" s="57" t="s">
+      <c r="B29" s="59"/>
+      <c r="C29" s="59"/>
+      <c r="D29" s="59"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="59"/>
+      <c r="G29" s="59"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="59"/>
+      <c r="K29" s="59"/>
+      <c r="L29" s="59"/>
+      <c r="M29" s="59"/>
+      <c r="N29" s="59"/>
+      <c r="O29" s="60"/>
+      <c r="P29" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="P29" s="57"/>
-      <c r="Q29" s="58"/>
-      <c r="R29" s="19"/>
-    </row>
-    <row r="30" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="68"/>
-      <c r="B30" s="69"/>
-      <c r="C30" s="69"/>
-      <c r="D30" s="69"/>
-      <c r="E30" s="69"/>
-      <c r="F30" s="69"/>
-      <c r="G30" s="69"/>
-      <c r="H30" s="69"/>
-      <c r="I30" s="69"/>
-      <c r="J30" s="69"/>
-      <c r="K30" s="69"/>
-      <c r="L30" s="69"/>
-      <c r="M30" s="69"/>
-      <c r="N30" s="70"/>
-      <c r="O30" s="59"/>
-      <c r="P30" s="59"/>
-      <c r="Q30" s="60"/>
-      <c r="R30" s="19"/>
-    </row>
-    <row r="31" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q29" s="50"/>
+      <c r="R29" s="51"/>
+      <c r="S29" s="19"/>
+    </row>
+    <row r="30" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="61"/>
+      <c r="B30" s="62"/>
+      <c r="C30" s="62"/>
+      <c r="D30" s="62"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="62"/>
+      <c r="G30" s="62"/>
+      <c r="H30" s="62"/>
+      <c r="I30" s="62"/>
+      <c r="J30" s="62"/>
+      <c r="K30" s="62"/>
+      <c r="L30" s="62"/>
+      <c r="M30" s="62"/>
+      <c r="N30" s="62"/>
+      <c r="O30" s="63"/>
+      <c r="P30" s="52"/>
+      <c r="Q30" s="52"/>
+      <c r="R30" s="53"/>
+      <c r="S30" s="19"/>
+    </row>
+    <row r="31" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
         <v>11</v>
       </c>
@@ -1876,646 +1880,677 @@
       <c r="D31" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E31" s="62" t="s">
+      <c r="E31" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="F31" s="63"/>
-      <c r="G31" s="63"/>
-      <c r="H31" s="63"/>
-      <c r="I31" s="63"/>
-      <c r="J31" s="63"/>
-      <c r="K31" s="63"/>
-      <c r="L31" s="63"/>
-      <c r="M31" s="63"/>
-      <c r="N31" s="64"/>
-      <c r="O31" s="61"/>
-      <c r="P31" s="61"/>
-      <c r="Q31" s="41"/>
-      <c r="R31" s="19"/>
-    </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="F31" s="56"/>
+      <c r="G31" s="56"/>
+      <c r="H31" s="56"/>
+      <c r="I31" s="56"/>
+      <c r="J31" s="56"/>
+      <c r="K31" s="56"/>
+      <c r="L31" s="56"/>
+      <c r="M31" s="56"/>
+      <c r="N31" s="56"/>
+      <c r="O31" s="57"/>
+      <c r="P31" s="54"/>
+      <c r="Q31" s="54"/>
+      <c r="R31" s="37"/>
+      <c r="S31" s="19"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="8"/>
       <c r="B32" s="23"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
-      <c r="E32" s="71"/>
-      <c r="F32" s="71"/>
-      <c r="G32" s="71"/>
+      <c r="E32" s="64"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="64"/>
       <c r="H32" s="6"/>
       <c r="I32" s="6"/>
       <c r="J32" s="9"/>
-      <c r="K32" s="42"/>
-      <c r="L32" s="43"/>
-      <c r="M32" s="22"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="48"/>
-      <c r="P32" s="48"/>
-      <c r="Q32" s="49"/>
-      <c r="R32" s="18"/>
-    </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K32" s="9"/>
+      <c r="L32" s="38"/>
+      <c r="M32" s="39"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="44"/>
+      <c r="Q32" s="44"/>
+      <c r="R32" s="45"/>
+      <c r="S32" s="18"/>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="24"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
-      <c r="E33" s="72"/>
-      <c r="F33" s="72"/>
-      <c r="G33" s="72"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="65"/>
+      <c r="G33" s="65"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
       <c r="J33" s="5"/>
-      <c r="K33" s="44"/>
-      <c r="L33" s="45"/>
-      <c r="M33" s="21"/>
-      <c r="N33" s="3"/>
-      <c r="O33" s="50"/>
-      <c r="P33" s="50"/>
-      <c r="Q33" s="51"/>
-      <c r="R33" s="18"/>
-    </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K33" s="5"/>
+      <c r="L33" s="40"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="21"/>
+      <c r="O33" s="3"/>
+      <c r="P33" s="46"/>
+      <c r="Q33" s="46"/>
+      <c r="R33" s="47"/>
+      <c r="S33" s="18"/>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
       <c r="B34" s="24"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
-      <c r="E34" s="72"/>
-      <c r="F34" s="72"/>
-      <c r="G34" s="72"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="65"/>
+      <c r="G34" s="65"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
       <c r="J34" s="5"/>
-      <c r="K34" s="44"/>
-      <c r="L34" s="45"/>
-      <c r="M34" s="21"/>
-      <c r="N34" s="3"/>
-      <c r="O34" s="50"/>
-      <c r="P34" s="50"/>
-      <c r="Q34" s="51"/>
-      <c r="R34" s="18"/>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K34" s="5"/>
+      <c r="L34" s="40"/>
+      <c r="M34" s="41"/>
+      <c r="N34" s="21"/>
+      <c r="O34" s="3"/>
+      <c r="P34" s="46"/>
+      <c r="Q34" s="46"/>
+      <c r="R34" s="47"/>
+      <c r="S34" s="18"/>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="24"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
-      <c r="E35" s="72"/>
-      <c r="F35" s="72"/>
-      <c r="G35" s="72"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
       <c r="J35" s="5"/>
-      <c r="K35" s="44"/>
-      <c r="L35" s="45"/>
-      <c r="M35" s="21"/>
-      <c r="N35" s="3"/>
-      <c r="O35" s="50"/>
-      <c r="P35" s="50"/>
-      <c r="Q35" s="51"/>
-      <c r="R35" s="18"/>
-    </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K35" s="5"/>
+      <c r="L35" s="40"/>
+      <c r="M35" s="41"/>
+      <c r="N35" s="21"/>
+      <c r="O35" s="3"/>
+      <c r="P35" s="46"/>
+      <c r="Q35" s="46"/>
+      <c r="R35" s="47"/>
+      <c r="S35" s="18"/>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
       <c r="B36" s="24"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
-      <c r="E36" s="72"/>
-      <c r="F36" s="72"/>
-      <c r="G36" s="72"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="65"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
       <c r="J36" s="5"/>
-      <c r="K36" s="44"/>
-      <c r="L36" s="45"/>
-      <c r="M36" s="21"/>
-      <c r="N36" s="3"/>
-      <c r="O36" s="50"/>
-      <c r="P36" s="50"/>
-      <c r="Q36" s="51"/>
-      <c r="R36" s="18"/>
-    </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K36" s="5"/>
+      <c r="L36" s="40"/>
+      <c r="M36" s="41"/>
+      <c r="N36" s="21"/>
+      <c r="O36" s="3"/>
+      <c r="P36" s="46"/>
+      <c r="Q36" s="46"/>
+      <c r="R36" s="47"/>
+      <c r="S36" s="18"/>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="24"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
-      <c r="E37" s="72"/>
-      <c r="F37" s="72"/>
-      <c r="G37" s="72"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
       <c r="J37" s="5"/>
-      <c r="K37" s="44"/>
-      <c r="L37" s="45"/>
-      <c r="M37" s="21"/>
-      <c r="N37" s="3"/>
-      <c r="O37" s="50"/>
-      <c r="P37" s="50"/>
-      <c r="Q37" s="51"/>
-      <c r="R37" s="18"/>
-    </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K37" s="5"/>
+      <c r="L37" s="40"/>
+      <c r="M37" s="41"/>
+      <c r="N37" s="21"/>
+      <c r="O37" s="3"/>
+      <c r="P37" s="46"/>
+      <c r="Q37" s="46"/>
+      <c r="R37" s="47"/>
+      <c r="S37" s="18"/>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="24"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
-      <c r="E38" s="72"/>
-      <c r="F38" s="72"/>
-      <c r="G38" s="72"/>
+      <c r="E38" s="65"/>
+      <c r="F38" s="65"/>
+      <c r="G38" s="65"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
       <c r="J38" s="5"/>
-      <c r="K38" s="44"/>
-      <c r="L38" s="45"/>
-      <c r="M38" s="21"/>
-      <c r="N38" s="3"/>
-      <c r="O38" s="50"/>
-      <c r="P38" s="50"/>
-      <c r="Q38" s="51"/>
-      <c r="R38" s="18"/>
-    </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K38" s="5"/>
+      <c r="L38" s="40"/>
+      <c r="M38" s="41"/>
+      <c r="N38" s="21"/>
+      <c r="O38" s="3"/>
+      <c r="P38" s="46"/>
+      <c r="Q38" s="46"/>
+      <c r="R38" s="47"/>
+      <c r="S38" s="18"/>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="10"/>
       <c r="B39" s="26"/>
       <c r="C39" s="7"/>
       <c r="D39" s="7"/>
-      <c r="E39" s="72"/>
-      <c r="F39" s="72"/>
-      <c r="G39" s="72"/>
+      <c r="E39" s="65"/>
+      <c r="F39" s="65"/>
+      <c r="G39" s="65"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="11"/>
-      <c r="K39" s="44"/>
-      <c r="L39" s="45"/>
-      <c r="M39" s="21"/>
-      <c r="N39" s="7"/>
-      <c r="O39" s="50"/>
-      <c r="P39" s="50"/>
-      <c r="Q39" s="51"/>
-      <c r="R39" s="18"/>
-    </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K39" s="11"/>
+      <c r="L39" s="40"/>
+      <c r="M39" s="41"/>
+      <c r="N39" s="21"/>
+      <c r="O39" s="7"/>
+      <c r="P39" s="46"/>
+      <c r="Q39" s="46"/>
+      <c r="R39" s="47"/>
+      <c r="S39" s="18"/>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40" s="10"/>
       <c r="B40" s="26"/>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
-      <c r="E40" s="72"/>
-      <c r="F40" s="72"/>
-      <c r="G40" s="72"/>
+      <c r="E40" s="65"/>
+      <c r="F40" s="65"/>
+      <c r="G40" s="65"/>
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
       <c r="J40" s="11"/>
-      <c r="K40" s="44"/>
-      <c r="L40" s="45"/>
-      <c r="M40" s="21"/>
-      <c r="N40" s="7"/>
-      <c r="O40" s="50"/>
-      <c r="P40" s="50"/>
-      <c r="Q40" s="51"/>
-      <c r="R40" s="18"/>
-    </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K40" s="11"/>
+      <c r="L40" s="40"/>
+      <c r="M40" s="41"/>
+      <c r="N40" s="21"/>
+      <c r="O40" s="7"/>
+      <c r="P40" s="46"/>
+      <c r="Q40" s="46"/>
+      <c r="R40" s="47"/>
+      <c r="S40" s="18"/>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
       <c r="B41" s="26"/>
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
-      <c r="E41" s="72"/>
-      <c r="F41" s="72"/>
-      <c r="G41" s="72"/>
+      <c r="E41" s="65"/>
+      <c r="F41" s="65"/>
+      <c r="G41" s="65"/>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
       <c r="J41" s="11"/>
-      <c r="K41" s="44"/>
-      <c r="L41" s="45"/>
-      <c r="M41" s="21"/>
-      <c r="N41" s="7"/>
-      <c r="O41" s="50"/>
-      <c r="P41" s="50"/>
-      <c r="Q41" s="51"/>
-      <c r="R41" s="18"/>
-    </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K41" s="11"/>
+      <c r="L41" s="40"/>
+      <c r="M41" s="41"/>
+      <c r="N41" s="21"/>
+      <c r="O41" s="7"/>
+      <c r="P41" s="46"/>
+      <c r="Q41" s="46"/>
+      <c r="R41" s="47"/>
+      <c r="S41" s="18"/>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="7"/>
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
-      <c r="E42" s="50"/>
-      <c r="F42" s="50"/>
-      <c r="G42" s="50"/>
+      <c r="E42" s="46"/>
+      <c r="F42" s="46"/>
+      <c r="G42" s="46"/>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
       <c r="J42" s="7"/>
-      <c r="K42" s="44"/>
-      <c r="L42" s="45"/>
-      <c r="M42" s="21"/>
-      <c r="N42" s="7"/>
-      <c r="O42" s="50"/>
-      <c r="P42" s="50"/>
-      <c r="Q42" s="50"/>
-      <c r="R42" s="18"/>
-    </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K42" s="11"/>
+      <c r="L42" s="40"/>
+      <c r="M42" s="41"/>
+      <c r="N42" s="21"/>
+      <c r="O42" s="7"/>
+      <c r="P42" s="46"/>
+      <c r="Q42" s="46"/>
+      <c r="R42" s="46"/>
+      <c r="S42" s="18"/>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
       <c r="D43" s="7"/>
-      <c r="E43" s="50"/>
-      <c r="F43" s="50"/>
-      <c r="G43" s="50"/>
+      <c r="E43" s="46"/>
+      <c r="F43" s="46"/>
+      <c r="G43" s="46"/>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
       <c r="J43" s="7"/>
-      <c r="K43" s="44"/>
-      <c r="L43" s="45"/>
-      <c r="M43" s="21"/>
-      <c r="N43" s="7"/>
-      <c r="O43" s="50"/>
-      <c r="P43" s="50"/>
-      <c r="Q43" s="50"/>
-      <c r="R43" s="18"/>
-    </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K43" s="11"/>
+      <c r="L43" s="40"/>
+      <c r="M43" s="41"/>
+      <c r="N43" s="21"/>
+      <c r="O43" s="7"/>
+      <c r="P43" s="46"/>
+      <c r="Q43" s="46"/>
+      <c r="R43" s="46"/>
+      <c r="S43" s="18"/>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
-      <c r="E44" s="50"/>
-      <c r="F44" s="50"/>
-      <c r="G44" s="50"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
       <c r="H44" s="7"/>
       <c r="I44" s="7"/>
       <c r="J44" s="7"/>
-      <c r="K44" s="44"/>
-      <c r="L44" s="45"/>
-      <c r="M44" s="21"/>
-      <c r="N44" s="7"/>
-      <c r="O44" s="50"/>
-      <c r="P44" s="50"/>
-      <c r="Q44" s="50"/>
-      <c r="R44" s="18"/>
-    </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K44" s="11"/>
+      <c r="L44" s="40"/>
+      <c r="M44" s="41"/>
+      <c r="N44" s="21"/>
+      <c r="O44" s="7"/>
+      <c r="P44" s="46"/>
+      <c r="Q44" s="46"/>
+      <c r="R44" s="46"/>
+      <c r="S44" s="18"/>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="33"/>
-      <c r="G45" s="73"/>
+      <c r="E45" s="31"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="66"/>
       <c r="H45" s="7"/>
       <c r="I45" s="7"/>
       <c r="J45" s="7"/>
-      <c r="K45" s="44"/>
-      <c r="L45" s="45"/>
-      <c r="M45" s="21"/>
-      <c r="N45" s="7"/>
-      <c r="O45" s="50"/>
-      <c r="P45" s="50"/>
-      <c r="Q45" s="50"/>
-      <c r="R45" s="18"/>
-    </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K45" s="11"/>
+      <c r="L45" s="40"/>
+      <c r="M45" s="41"/>
+      <c r="N45" s="21"/>
+      <c r="O45" s="7"/>
+      <c r="P45" s="46"/>
+      <c r="Q45" s="46"/>
+      <c r="R45" s="46"/>
+      <c r="S45" s="18"/>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
-      <c r="E46" s="32"/>
-      <c r="F46" s="33"/>
-      <c r="G46" s="73"/>
+      <c r="E46" s="31"/>
+      <c r="F46" s="32"/>
+      <c r="G46" s="66"/>
       <c r="H46" s="7"/>
       <c r="I46" s="7"/>
       <c r="J46" s="7"/>
-      <c r="K46" s="44"/>
-      <c r="L46" s="45"/>
-      <c r="M46" s="21"/>
-      <c r="N46" s="7"/>
-      <c r="O46" s="50"/>
-      <c r="P46" s="50"/>
-      <c r="Q46" s="50"/>
-      <c r="R46" s="18"/>
-    </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K46" s="11"/>
+      <c r="L46" s="40"/>
+      <c r="M46" s="41"/>
+      <c r="N46" s="21"/>
+      <c r="O46" s="7"/>
+      <c r="P46" s="46"/>
+      <c r="Q46" s="46"/>
+      <c r="R46" s="46"/>
+      <c r="S46" s="18"/>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="32"/>
-      <c r="F47" s="33"/>
-      <c r="G47" s="73"/>
+      <c r="E47" s="31"/>
+      <c r="F47" s="32"/>
+      <c r="G47" s="66"/>
       <c r="H47" s="7"/>
       <c r="I47" s="7"/>
       <c r="J47" s="7"/>
-      <c r="K47" s="44"/>
-      <c r="L47" s="45"/>
-      <c r="M47" s="21"/>
-      <c r="N47" s="7"/>
-      <c r="O47" s="50"/>
-      <c r="P47" s="50"/>
-      <c r="Q47" s="50"/>
-      <c r="R47" s="18"/>
-    </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K47" s="11"/>
+      <c r="L47" s="40"/>
+      <c r="M47" s="41"/>
+      <c r="N47" s="21"/>
+      <c r="O47" s="7"/>
+      <c r="P47" s="46"/>
+      <c r="Q47" s="46"/>
+      <c r="R47" s="46"/>
+      <c r="S47" s="18"/>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
-      <c r="E48" s="32"/>
-      <c r="F48" s="33"/>
-      <c r="G48" s="73"/>
+      <c r="E48" s="31"/>
+      <c r="F48" s="32"/>
+      <c r="G48" s="66"/>
       <c r="H48" s="7"/>
       <c r="I48" s="7"/>
       <c r="J48" s="7"/>
-      <c r="K48" s="44"/>
-      <c r="L48" s="45"/>
-      <c r="M48" s="21"/>
-      <c r="N48" s="7"/>
-      <c r="O48" s="50"/>
-      <c r="P48" s="50"/>
-      <c r="Q48" s="50"/>
-      <c r="R48" s="18"/>
-    </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K48" s="11"/>
+      <c r="L48" s="40"/>
+      <c r="M48" s="41"/>
+      <c r="N48" s="21"/>
+      <c r="O48" s="7"/>
+      <c r="P48" s="46"/>
+      <c r="Q48" s="46"/>
+      <c r="R48" s="46"/>
+      <c r="S48" s="18"/>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="33"/>
-      <c r="G49" s="73"/>
+      <c r="E49" s="31"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="66"/>
       <c r="H49" s="7"/>
       <c r="I49" s="7"/>
       <c r="J49" s="7"/>
-      <c r="K49" s="44"/>
-      <c r="L49" s="45"/>
-      <c r="M49" s="21"/>
-      <c r="N49" s="7"/>
-      <c r="O49" s="50"/>
-      <c r="P49" s="50"/>
-      <c r="Q49" s="50"/>
-      <c r="R49" s="18"/>
-    </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K49" s="11"/>
+      <c r="L49" s="40"/>
+      <c r="M49" s="41"/>
+      <c r="N49" s="21"/>
+      <c r="O49" s="7"/>
+      <c r="P49" s="46"/>
+      <c r="Q49" s="46"/>
+      <c r="R49" s="46"/>
+      <c r="S49" s="18"/>
+    </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
       <c r="D50" s="7"/>
-      <c r="E50" s="32"/>
-      <c r="F50" s="33"/>
-      <c r="G50" s="73"/>
+      <c r="E50" s="31"/>
+      <c r="F50" s="32"/>
+      <c r="G50" s="66"/>
       <c r="H50" s="7"/>
       <c r="I50" s="7"/>
       <c r="J50" s="7"/>
-      <c r="K50" s="44"/>
-      <c r="L50" s="45"/>
-      <c r="M50" s="21"/>
-      <c r="N50" s="7"/>
-      <c r="O50" s="50"/>
-      <c r="P50" s="50"/>
-      <c r="Q50" s="50"/>
-      <c r="R50" s="18"/>
-    </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K50" s="11"/>
+      <c r="L50" s="40"/>
+      <c r="M50" s="41"/>
+      <c r="N50" s="21"/>
+      <c r="O50" s="7"/>
+      <c r="P50" s="46"/>
+      <c r="Q50" s="46"/>
+      <c r="R50" s="46"/>
+      <c r="S50" s="18"/>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
       <c r="B51" s="7"/>
       <c r="C51" s="7"/>
       <c r="D51" s="7"/>
-      <c r="E51" s="32"/>
-      <c r="F51" s="33"/>
-      <c r="G51" s="73"/>
+      <c r="E51" s="31"/>
+      <c r="F51" s="32"/>
+      <c r="G51" s="66"/>
       <c r="H51" s="7"/>
       <c r="I51" s="7"/>
       <c r="J51" s="7"/>
-      <c r="K51" s="44"/>
-      <c r="L51" s="45"/>
-      <c r="M51" s="21"/>
-      <c r="N51" s="7"/>
-      <c r="O51" s="50"/>
-      <c r="P51" s="50"/>
-      <c r="Q51" s="50"/>
-      <c r="R51" s="18"/>
-    </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K51" s="11"/>
+      <c r="L51" s="40"/>
+      <c r="M51" s="41"/>
+      <c r="N51" s="21"/>
+      <c r="O51" s="7"/>
+      <c r="P51" s="46"/>
+      <c r="Q51" s="46"/>
+      <c r="R51" s="46"/>
+      <c r="S51" s="18"/>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
-      <c r="E52" s="32"/>
-      <c r="F52" s="33"/>
-      <c r="G52" s="73"/>
+      <c r="E52" s="31"/>
+      <c r="F52" s="32"/>
+      <c r="G52" s="66"/>
       <c r="H52" s="7"/>
       <c r="I52" s="7"/>
       <c r="J52" s="7"/>
-      <c r="K52" s="44"/>
-      <c r="L52" s="45"/>
-      <c r="M52" s="21"/>
-      <c r="N52" s="7"/>
-      <c r="O52" s="50"/>
-      <c r="P52" s="50"/>
-      <c r="Q52" s="50"/>
-      <c r="R52" s="18"/>
-    </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K52" s="11"/>
+      <c r="L52" s="40"/>
+      <c r="M52" s="41"/>
+      <c r="N52" s="21"/>
+      <c r="O52" s="7"/>
+      <c r="P52" s="46"/>
+      <c r="Q52" s="46"/>
+      <c r="R52" s="46"/>
+      <c r="S52" s="18"/>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="7"/>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
-      <c r="E53" s="32"/>
-      <c r="F53" s="33"/>
-      <c r="G53" s="73"/>
+      <c r="E53" s="31"/>
+      <c r="F53" s="32"/>
+      <c r="G53" s="66"/>
       <c r="H53" s="7"/>
       <c r="I53" s="7"/>
       <c r="J53" s="7"/>
-      <c r="K53" s="44"/>
-      <c r="L53" s="45"/>
-      <c r="M53" s="21"/>
-      <c r="N53" s="7"/>
-      <c r="O53" s="50"/>
-      <c r="P53" s="50"/>
-      <c r="Q53" s="50"/>
-      <c r="R53" s="18"/>
-    </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K53" s="11"/>
+      <c r="L53" s="40"/>
+      <c r="M53" s="41"/>
+      <c r="N53" s="21"/>
+      <c r="O53" s="7"/>
+      <c r="P53" s="46"/>
+      <c r="Q53" s="46"/>
+      <c r="R53" s="46"/>
+      <c r="S53" s="18"/>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
-      <c r="E54" s="32"/>
-      <c r="F54" s="33"/>
-      <c r="G54" s="73"/>
+      <c r="E54" s="31"/>
+      <c r="F54" s="32"/>
+      <c r="G54" s="66"/>
       <c r="H54" s="7"/>
       <c r="I54" s="7"/>
       <c r="J54" s="7"/>
-      <c r="K54" s="44"/>
-      <c r="L54" s="45"/>
-      <c r="M54" s="21"/>
-      <c r="N54" s="7"/>
-      <c r="O54" s="50"/>
-      <c r="P54" s="50"/>
-      <c r="Q54" s="50"/>
-      <c r="R54" s="18"/>
-    </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K54" s="11"/>
+      <c r="L54" s="40"/>
+      <c r="M54" s="41"/>
+      <c r="N54" s="21"/>
+      <c r="O54" s="7"/>
+      <c r="P54" s="46"/>
+      <c r="Q54" s="46"/>
+      <c r="R54" s="46"/>
+      <c r="S54" s="18"/>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="32"/>
-      <c r="F55" s="33"/>
-      <c r="G55" s="73"/>
+      <c r="E55" s="31"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="66"/>
       <c r="H55" s="7"/>
       <c r="I55" s="7"/>
       <c r="J55" s="7"/>
-      <c r="K55" s="44"/>
-      <c r="L55" s="45"/>
-      <c r="M55" s="21"/>
-      <c r="N55" s="7"/>
-      <c r="O55" s="50"/>
-      <c r="P55" s="50"/>
-      <c r="Q55" s="50"/>
-      <c r="R55" s="18"/>
-    </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K55" s="11"/>
+      <c r="L55" s="40"/>
+      <c r="M55" s="41"/>
+      <c r="N55" s="21"/>
+      <c r="O55" s="7"/>
+      <c r="P55" s="46"/>
+      <c r="Q55" s="46"/>
+      <c r="R55" s="46"/>
+      <c r="S55" s="18"/>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
       <c r="B56" s="7"/>
       <c r="C56" s="7"/>
       <c r="D56" s="7"/>
-      <c r="E56" s="32"/>
-      <c r="F56" s="33"/>
-      <c r="G56" s="73"/>
+      <c r="E56" s="31"/>
+      <c r="F56" s="32"/>
+      <c r="G56" s="66"/>
       <c r="H56" s="7"/>
       <c r="I56" s="7"/>
       <c r="J56" s="7"/>
-      <c r="K56" s="44"/>
-      <c r="L56" s="45"/>
-      <c r="M56" s="21"/>
-      <c r="N56" s="7"/>
-      <c r="O56" s="50"/>
-      <c r="P56" s="50"/>
-      <c r="Q56" s="50"/>
-      <c r="R56" s="18"/>
-    </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K56" s="11"/>
+      <c r="L56" s="40"/>
+      <c r="M56" s="41"/>
+      <c r="N56" s="21"/>
+      <c r="O56" s="7"/>
+      <c r="P56" s="46"/>
+      <c r="Q56" s="46"/>
+      <c r="R56" s="46"/>
+      <c r="S56" s="18"/>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
       <c r="B57" s="7"/>
       <c r="C57" s="7"/>
       <c r="D57" s="7"/>
-      <c r="E57" s="32"/>
-      <c r="F57" s="33"/>
-      <c r="G57" s="73"/>
+      <c r="E57" s="31"/>
+      <c r="F57" s="32"/>
+      <c r="G57" s="66"/>
       <c r="H57" s="7"/>
       <c r="I57" s="7"/>
       <c r="J57" s="7"/>
-      <c r="K57" s="44"/>
-      <c r="L57" s="45"/>
-      <c r="M57" s="21"/>
-      <c r="N57" s="7"/>
-      <c r="O57" s="50"/>
-      <c r="P57" s="50"/>
-      <c r="Q57" s="50"/>
-      <c r="R57" s="18"/>
-    </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K57" s="11"/>
+      <c r="L57" s="40"/>
+      <c r="M57" s="41"/>
+      <c r="N57" s="21"/>
+      <c r="O57" s="7"/>
+      <c r="P57" s="46"/>
+      <c r="Q57" s="46"/>
+      <c r="R57" s="46"/>
+      <c r="S57" s="18"/>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
       <c r="B58" s="7"/>
       <c r="C58" s="7"/>
       <c r="D58" s="7"/>
-      <c r="E58" s="32"/>
-      <c r="F58" s="33"/>
-      <c r="G58" s="73"/>
+      <c r="E58" s="31"/>
+      <c r="F58" s="32"/>
+      <c r="G58" s="66"/>
       <c r="H58" s="7"/>
       <c r="I58" s="7"/>
       <c r="J58" s="7"/>
-      <c r="K58" s="44"/>
-      <c r="L58" s="45"/>
-      <c r="M58" s="21"/>
-      <c r="N58" s="7"/>
-      <c r="O58" s="50"/>
-      <c r="P58" s="50"/>
-      <c r="Q58" s="50"/>
-      <c r="R58" s="18"/>
-    </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K58" s="11"/>
+      <c r="L58" s="40"/>
+      <c r="M58" s="41"/>
+      <c r="N58" s="21"/>
+      <c r="O58" s="7"/>
+      <c r="P58" s="46"/>
+      <c r="Q58" s="46"/>
+      <c r="R58" s="46"/>
+      <c r="S58" s="18"/>
+    </row>
+    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
       <c r="B59" s="7"/>
       <c r="C59" s="7"/>
       <c r="D59" s="7"/>
-      <c r="E59" s="32"/>
-      <c r="F59" s="33"/>
-      <c r="G59" s="73"/>
+      <c r="E59" s="31"/>
+      <c r="F59" s="32"/>
+      <c r="G59" s="66"/>
       <c r="H59" s="7"/>
       <c r="I59" s="7"/>
       <c r="J59" s="7"/>
-      <c r="K59" s="44"/>
-      <c r="L59" s="45"/>
-      <c r="M59" s="21"/>
-      <c r="N59" s="7"/>
-      <c r="O59" s="50"/>
-      <c r="P59" s="50"/>
-      <c r="Q59" s="50"/>
-      <c r="R59" s="18"/>
-    </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K59" s="11"/>
+      <c r="L59" s="40"/>
+      <c r="M59" s="41"/>
+      <c r="N59" s="21"/>
+      <c r="O59" s="7"/>
+      <c r="P59" s="46"/>
+      <c r="Q59" s="46"/>
+      <c r="R59" s="46"/>
+      <c r="S59" s="18"/>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
       <c r="B60" s="7"/>
       <c r="C60" s="7"/>
       <c r="D60" s="7"/>
-      <c r="E60" s="32"/>
-      <c r="F60" s="33"/>
-      <c r="G60" s="73"/>
+      <c r="E60" s="31"/>
+      <c r="F60" s="32"/>
+      <c r="G60" s="66"/>
       <c r="H60" s="7"/>
       <c r="I60" s="7"/>
       <c r="J60" s="7"/>
-      <c r="K60" s="44"/>
-      <c r="L60" s="45"/>
-      <c r="M60" s="21"/>
-      <c r="N60" s="7"/>
-      <c r="O60" s="50"/>
-      <c r="P60" s="50"/>
-      <c r="Q60" s="50"/>
-      <c r="R60" s="18"/>
+      <c r="K60" s="11"/>
+      <c r="L60" s="40"/>
+      <c r="M60" s="41"/>
+      <c r="N60" s="21"/>
+      <c r="O60" s="7"/>
+      <c r="P60" s="46"/>
+      <c r="Q60" s="46"/>
+      <c r="R60" s="46"/>
+      <c r="S60" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="143">
-    <mergeCell ref="K57:L57"/>
-    <mergeCell ref="K58:L58"/>
-    <mergeCell ref="K59:L59"/>
-    <mergeCell ref="K60:L60"/>
-    <mergeCell ref="K46:L46"/>
-    <mergeCell ref="K47:L47"/>
-    <mergeCell ref="K48:L48"/>
-    <mergeCell ref="K49:L49"/>
-    <mergeCell ref="K50:L50"/>
-    <mergeCell ref="K51:L51"/>
-    <mergeCell ref="K52:L52"/>
-    <mergeCell ref="K53:L53"/>
-    <mergeCell ref="K54:L54"/>
-    <mergeCell ref="K55:L55"/>
-    <mergeCell ref="K56:L56"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="K38:L38"/>
-    <mergeCell ref="K39:L39"/>
-    <mergeCell ref="K40:L40"/>
-    <mergeCell ref="K41:L41"/>
-    <mergeCell ref="K42:L42"/>
-    <mergeCell ref="K43:L43"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="O56:Q56"/>
-    <mergeCell ref="O57:Q57"/>
-    <mergeCell ref="O58:Q58"/>
-    <mergeCell ref="O59:Q59"/>
-    <mergeCell ref="O60:Q60"/>
-    <mergeCell ref="O43:Q43"/>
-    <mergeCell ref="O44:Q44"/>
-    <mergeCell ref="O45:Q45"/>
-    <mergeCell ref="O46:Q46"/>
-    <mergeCell ref="O47:Q47"/>
-    <mergeCell ref="O48:Q48"/>
-    <mergeCell ref="O49:Q49"/>
-    <mergeCell ref="O50:Q50"/>
-    <mergeCell ref="O51:Q51"/>
-    <mergeCell ref="O52:Q52"/>
-    <mergeCell ref="O53:Q53"/>
-    <mergeCell ref="O54:Q54"/>
-    <mergeCell ref="O55:Q55"/>
+  <mergeCells count="141">
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="L57:M57"/>
+    <mergeCell ref="L58:M58"/>
+    <mergeCell ref="L59:M59"/>
+    <mergeCell ref="L60:M60"/>
+    <mergeCell ref="L46:M46"/>
+    <mergeCell ref="L47:M47"/>
+    <mergeCell ref="L48:M48"/>
+    <mergeCell ref="L49:M49"/>
+    <mergeCell ref="L50:M50"/>
+    <mergeCell ref="L51:M51"/>
+    <mergeCell ref="L52:M52"/>
+    <mergeCell ref="L53:M53"/>
+    <mergeCell ref="L54:M54"/>
+    <mergeCell ref="L55:M55"/>
+    <mergeCell ref="L56:M56"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="P56:R56"/>
+    <mergeCell ref="P57:R57"/>
+    <mergeCell ref="P58:R58"/>
+    <mergeCell ref="P59:R59"/>
+    <mergeCell ref="P60:R60"/>
+    <mergeCell ref="P43:R43"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="P45:R45"/>
+    <mergeCell ref="P46:R46"/>
+    <mergeCell ref="P47:R47"/>
+    <mergeCell ref="P48:R48"/>
+    <mergeCell ref="P49:R49"/>
+    <mergeCell ref="P50:R50"/>
+    <mergeCell ref="P51:R51"/>
+    <mergeCell ref="P52:R52"/>
+    <mergeCell ref="P53:R53"/>
+    <mergeCell ref="P54:R54"/>
+    <mergeCell ref="P55:R55"/>
     <mergeCell ref="E57:G57"/>
     <mergeCell ref="E58:G58"/>
     <mergeCell ref="E59:G59"/>
@@ -2527,9 +2562,9 @@
     <mergeCell ref="E55:G55"/>
     <mergeCell ref="E56:G56"/>
     <mergeCell ref="E38:G38"/>
-    <mergeCell ref="O38:Q38"/>
-    <mergeCell ref="O39:Q39"/>
-    <mergeCell ref="O40:Q40"/>
+    <mergeCell ref="P38:R38"/>
+    <mergeCell ref="P39:R39"/>
+    <mergeCell ref="P40:R40"/>
     <mergeCell ref="E48:G48"/>
     <mergeCell ref="E49:G49"/>
     <mergeCell ref="E50:G50"/>
@@ -2537,47 +2572,47 @@
     <mergeCell ref="E43:G43"/>
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="E45:G45"/>
-    <mergeCell ref="O41:Q41"/>
-    <mergeCell ref="O42:Q42"/>
-    <mergeCell ref="K45:L45"/>
+    <mergeCell ref="P41:R41"/>
+    <mergeCell ref="P42:R42"/>
+    <mergeCell ref="L45:M45"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="E40:G40"/>
     <mergeCell ref="E41:G41"/>
     <mergeCell ref="E46:G46"/>
     <mergeCell ref="E47:G47"/>
-    <mergeCell ref="O29:Q31"/>
-    <mergeCell ref="O37:Q37"/>
-    <mergeCell ref="O35:Q35"/>
-    <mergeCell ref="O36:Q36"/>
-    <mergeCell ref="E31:N31"/>
-    <mergeCell ref="A29:N30"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="O12:Q12"/>
+    <mergeCell ref="P29:R31"/>
+    <mergeCell ref="P37:R37"/>
+    <mergeCell ref="P35:R35"/>
+    <mergeCell ref="P36:R36"/>
+    <mergeCell ref="E31:O31"/>
+    <mergeCell ref="A29:O30"/>
+    <mergeCell ref="P27:R27"/>
+    <mergeCell ref="P28:R28"/>
+    <mergeCell ref="P12:R12"/>
     <mergeCell ref="E32:G32"/>
-    <mergeCell ref="O32:Q32"/>
+    <mergeCell ref="P32:R32"/>
     <mergeCell ref="E35:G35"/>
     <mergeCell ref="E36:G36"/>
     <mergeCell ref="E37:G37"/>
     <mergeCell ref="E33:G33"/>
-    <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="O34:Q34"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="P33:R33"/>
+    <mergeCell ref="P34:R34"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="L36:M36"/>
     <mergeCell ref="E34:G34"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="O13:Q13"/>
-    <mergeCell ref="O14:Q14"/>
-    <mergeCell ref="O15:Q15"/>
-    <mergeCell ref="O16:Q16"/>
-    <mergeCell ref="O7:Q7"/>
-    <mergeCell ref="O8:Q8"/>
-    <mergeCell ref="O9:Q9"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="O11:Q11"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="P14:R14"/>
+    <mergeCell ref="P15:R15"/>
+    <mergeCell ref="P16:R16"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="P9:R9"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="P11:R11"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C13:D13"/>
@@ -2594,20 +2629,17 @@
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E28:F28"/>
-    <mergeCell ref="O26:Q26"/>
+    <mergeCell ref="P26:R26"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="M2:N2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="O3:Q3"/>
-    <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="O6:Q6"/>
-    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="P6:R6"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="E4:F4"/>

</xml_diff>